<commit_message>
merge signle catgeory to atleast two suiatble catgeories
</commit_message>
<xml_diff>
--- a/Extracted_Data(MAS).xlsx
+++ b/Extracted_Data(MAS).xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="179">
   <si>
     <t>#ID</t>
   </si>
@@ -267,12 +267,15 @@
     <t>Category</t>
   </si>
   <si>
+    <t>Agent Runtime Problem (18)</t>
+  </si>
+  <si>
+    <t>Agent Lifecycle Problem (56)</t>
+  </si>
+  <si>
     <t>Agent Creation Problem (38)</t>
   </si>
   <si>
-    <t>Agent Initialization Problem (38)</t>
-  </si>
-  <si>
     <t>Handoff Problem (4)</t>
   </si>
   <si>
@@ -327,18 +330,15 @@
     <t>Missing Documentation (5)</t>
   </si>
   <si>
-    <t>Error Propagation Problem (18)</t>
-  </si>
-  <si>
-    <t>Error Handling Problem (18)</t>
+    <t>Frontend Problem (3)</t>
+  </si>
+  <si>
+    <t>Infrastructure Problem (9)</t>
   </si>
   <si>
     <t>Deployment Problem (3)</t>
   </si>
   <si>
-    <t>Infrastructure Problem (6)</t>
-  </si>
-  <si>
     <t>File System Handling Problem (1)</t>
   </si>
   <si>
@@ -405,12 +405,6 @@
     <t>Tool Schema Problem (13)</t>
   </si>
   <si>
-    <t>Frontend Problem (3)</t>
-  </si>
-  <si>
-    <t>UI/UX Problem (3)</t>
-  </si>
-  <si>
     <t>Context Management Problem (10)</t>
   </si>
   <si>
@@ -472,12 +466,6 @@
   </si>
   <si>
     <t>Update Environment Configuration (13)</t>
-  </si>
-  <si>
-    <t>Improve Frontend (3)</t>
-  </si>
-  <si>
-    <t>Enhance UI/UX (3)</t>
   </si>
   <si>
     <t>Enhance Exception Handling (19)</t>
@@ -520,10 +508,13 @@
     <t>Optimize Message Handling (17)</t>
   </si>
   <si>
+    <t>Improve Frontend (3)</t>
+  </si>
+  <si>
+    <t>Optimize Infrastructure (50)</t>
+  </si>
+  <si>
     <t>Database Compatibility (6)</t>
-  </si>
-  <si>
-    <t>Optimize Infrastructure (27)</t>
   </si>
   <si>
     <t>Optimize Memory Management (41)</t>
@@ -2666,9 +2657,7 @@
       <c r="B3" t="s" s="6">
         <v>86</v>
       </c>
-      <c r="C3" t="s" s="7">
-        <v>87</v>
-      </c>
+      <c r="C3" s="11"/>
       <c r="D3" s="3"/>
       <c r="E3" s="4"/>
     </row>
@@ -2677,9 +2666,11 @@
         <v>3</v>
       </c>
       <c r="B4" t="s" s="6">
+        <v>87</v>
+      </c>
+      <c r="C4" t="s" s="7">
         <v>88</v>
       </c>
-      <c r="C4" s="13"/>
       <c r="D4" s="3"/>
       <c r="E4" s="4"/>
     </row>
@@ -2701,9 +2692,7 @@
       <c r="B6" t="s" s="6">
         <v>90</v>
       </c>
-      <c r="C6" t="s" s="7">
-        <v>91</v>
-      </c>
+      <c r="C6" s="13"/>
       <c r="D6" s="3"/>
       <c r="E6" s="4"/>
     </row>
@@ -2712,9 +2701,11 @@
         <v>6</v>
       </c>
       <c r="B7" t="s" s="6">
+        <v>91</v>
+      </c>
+      <c r="C7" t="s" s="7">
         <v>92</v>
       </c>
-      <c r="C7" s="13"/>
       <c r="D7" s="3"/>
       <c r="E7" s="4"/>
     </row>
@@ -2725,9 +2716,7 @@
       <c r="B8" t="s" s="6">
         <v>93</v>
       </c>
-      <c r="C8" t="s" s="7">
-        <v>94</v>
-      </c>
+      <c r="C8" s="13"/>
       <c r="D8" s="3"/>
       <c r="E8" s="4"/>
     </row>
@@ -2736,9 +2725,11 @@
         <v>8</v>
       </c>
       <c r="B9" t="s" s="6">
+        <v>94</v>
+      </c>
+      <c r="C9" t="s" s="7">
         <v>95</v>
       </c>
-      <c r="C9" s="13"/>
       <c r="D9" s="3"/>
       <c r="E9" s="4"/>
     </row>
@@ -2760,9 +2751,7 @@
       <c r="B11" t="s" s="6">
         <v>97</v>
       </c>
-      <c r="C11" t="s" s="7">
-        <v>98</v>
-      </c>
+      <c r="C11" s="13"/>
       <c r="D11" s="3"/>
       <c r="E11" s="4"/>
     </row>
@@ -2771,9 +2760,11 @@
         <v>11</v>
       </c>
       <c r="B12" t="s" s="6">
+        <v>98</v>
+      </c>
+      <c r="C12" t="s" s="7">
         <v>99</v>
       </c>
-      <c r="C12" s="13"/>
       <c r="D12" s="3"/>
       <c r="E12" s="4"/>
     </row>
@@ -2795,9 +2786,7 @@
       <c r="B14" t="s" s="6">
         <v>101</v>
       </c>
-      <c r="C14" t="s" s="7">
-        <v>102</v>
-      </c>
+      <c r="C14" s="13"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
     </row>
@@ -2806,9 +2795,11 @@
         <v>14</v>
       </c>
       <c r="B15" t="s" s="6">
+        <v>102</v>
+      </c>
+      <c r="C15" t="s" s="7">
         <v>103</v>
       </c>
-      <c r="C15" s="13"/>
       <c r="D15" s="3"/>
       <c r="E15" s="4"/>
     </row>
@@ -2819,9 +2810,7 @@
       <c r="B16" t="s" s="6">
         <v>104</v>
       </c>
-      <c r="C16" t="s" s="7">
-        <v>105</v>
-      </c>
+      <c r="C16" s="13"/>
       <c r="D16" s="3"/>
       <c r="E16" s="4"/>
     </row>
@@ -2830,10 +2819,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s" s="6">
+        <v>105</v>
+      </c>
+      <c r="C17" t="s" s="7">
         <v>106</v>
-      </c>
-      <c r="C17" t="s" s="7">
-        <v>107</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="4"/>
@@ -2843,9 +2832,9 @@
         <v>17</v>
       </c>
       <c r="B18" t="s" s="6">
-        <v>108</v>
-      </c>
-      <c r="C18" s="13"/>
+        <v>107</v>
+      </c>
+      <c r="C18" s="11"/>
       <c r="D18" s="3"/>
       <c r="E18" s="4"/>
     </row>
@@ -2854,9 +2843,9 @@
         <v>18</v>
       </c>
       <c r="B19" t="s" s="6">
-        <v>109</v>
-      </c>
-      <c r="C19" s="13"/>
+        <v>108</v>
+      </c>
+      <c r="C19" s="11"/>
       <c r="D19" s="3"/>
       <c r="E19" s="4"/>
     </row>
@@ -2865,11 +2854,9 @@
         <v>19</v>
       </c>
       <c r="B20" t="s" s="6">
-        <v>110</v>
-      </c>
-      <c r="C20" t="s" s="7">
-        <v>111</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="C20" s="11"/>
       <c r="D20" s="3"/>
       <c r="E20" s="4"/>
     </row>
@@ -2878,18 +2865,20 @@
         <v>20</v>
       </c>
       <c r="B21" t="s" s="6">
-        <v>112</v>
-      </c>
-      <c r="C21" s="13"/>
+        <v>110</v>
+      </c>
+      <c r="C21" t="s" s="7">
+        <v>111</v>
+      </c>
       <c r="D21" s="3"/>
       <c r="E21" s="4"/>
     </row>
-    <row r="22" ht="12.6" customHeight="1">
+    <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="5">
         <v>21</v>
       </c>
       <c r="B22" t="s" s="6">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="3"/>
@@ -2900,11 +2889,9 @@
         <v>22</v>
       </c>
       <c r="B23" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C23" t="s" s="7">
-        <v>115</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="C23" s="13"/>
       <c r="D23" s="3"/>
       <c r="E23" s="4"/>
     </row>
@@ -2913,9 +2900,11 @@
         <v>23</v>
       </c>
       <c r="B24" t="s" s="6">
-        <v>116</v>
-      </c>
-      <c r="C24" s="13"/>
+        <v>114</v>
+      </c>
+      <c r="C24" t="s" s="7">
+        <v>115</v>
+      </c>
       <c r="D24" s="3"/>
       <c r="E24" s="4"/>
     </row>
@@ -2924,11 +2913,9 @@
         <v>24</v>
       </c>
       <c r="B25" t="s" s="6">
-        <v>117</v>
-      </c>
-      <c r="C25" t="s" s="7">
-        <v>118</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="C25" s="13"/>
       <c r="D25" s="3"/>
       <c r="E25" s="4"/>
     </row>
@@ -2937,9 +2924,11 @@
         <v>25</v>
       </c>
       <c r="B26" t="s" s="6">
-        <v>119</v>
-      </c>
-      <c r="C26" s="13"/>
+        <v>117</v>
+      </c>
+      <c r="C26" t="s" s="7">
+        <v>118</v>
+      </c>
       <c r="D26" s="3"/>
       <c r="E26" s="4"/>
     </row>
@@ -2948,7 +2937,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s" s="6">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="3"/>
@@ -2959,7 +2948,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s" s="6">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="3"/>
@@ -2970,11 +2959,9 @@
         <v>28</v>
       </c>
       <c r="B29" t="s" s="6">
-        <v>122</v>
-      </c>
-      <c r="C29" t="s" s="7">
-        <v>123</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="C29" s="13"/>
       <c r="D29" s="3"/>
       <c r="E29" s="4"/>
     </row>
@@ -2983,9 +2970,11 @@
         <v>29</v>
       </c>
       <c r="B30" t="s" s="6">
-        <v>124</v>
-      </c>
-      <c r="C30" s="13"/>
+        <v>122</v>
+      </c>
+      <c r="C30" t="s" s="7">
+        <v>123</v>
+      </c>
       <c r="D30" s="3"/>
       <c r="E30" s="4"/>
     </row>
@@ -2994,11 +2983,9 @@
         <v>30</v>
       </c>
       <c r="B31" t="s" s="6">
-        <v>125</v>
-      </c>
-      <c r="C31" t="s" s="7">
-        <v>126</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="C31" s="13"/>
       <c r="D31" s="3"/>
       <c r="E31" s="4"/>
     </row>
@@ -3007,9 +2994,11 @@
         <v>31</v>
       </c>
       <c r="B32" t="s" s="6">
-        <v>127</v>
-      </c>
-      <c r="C32" s="13"/>
+        <v>125</v>
+      </c>
+      <c r="C32" t="s" s="7">
+        <v>126</v>
+      </c>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
     </row>
@@ -3018,7 +3007,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s" s="6">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C33" s="13"/>
       <c r="D33" s="3"/>
@@ -3029,7 +3018,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s" s="6">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C34" s="13"/>
       <c r="D34" s="3"/>
@@ -3040,11 +3029,9 @@
         <v>34</v>
       </c>
       <c r="B35" t="s" s="6">
-        <v>130</v>
-      </c>
-      <c r="C35" t="s" s="7">
-        <v>131</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="C35" s="13"/>
       <c r="D35" s="3"/>
       <c r="E35" s="4"/>
     </row>
@@ -3053,10 +3040,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s" s="6">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C36" t="s" s="7">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="4"/>
@@ -3066,7 +3053,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s" s="6">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C37" s="13"/>
       <c r="D37" s="3"/>
@@ -3077,7 +3064,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s" s="6">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C38" s="13"/>
       <c r="D38" s="3"/>
@@ -3088,7 +3075,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s" s="6">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C39" s="13"/>
       <c r="D39" s="3"/>
@@ -3099,7 +3086,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s" s="6">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C40" s="13"/>
       <c r="D40" s="3"/>
@@ -3110,7 +3097,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s" s="6">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C41" s="13"/>
       <c r="D41" s="3"/>
@@ -3121,7 +3108,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s" s="6">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C42" s="13"/>
       <c r="D42" s="3"/>
@@ -3132,7 +3119,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s" s="6">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C43" s="13"/>
       <c r="D43" s="3"/>
@@ -3143,7 +3130,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s" s="6">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C44" s="13"/>
       <c r="D44" s="3"/>
@@ -3154,7 +3141,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s" s="6">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C45" s="13"/>
       <c r="D45" s="3"/>
@@ -3165,26 +3152,27 @@
         <v>45</v>
       </c>
       <c r="B46" t="s" s="14">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C46" s="13"/>
       <c r="D46" s="3"/>
       <c r="E46" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="C25:C28"/>
-    <mergeCell ref="C3:C5"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C8:C10"/>
+  <mergeCells count="13">
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C9:C11"/>
     <mergeCell ref="C36:C46"/>
-    <mergeCell ref="C31:C34"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="C32:C35"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="C21:C23"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C17:C20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
@@ -3224,10 +3212,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s" s="6">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C2" t="s" s="7">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
@@ -3237,7 +3225,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="6">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="3"/>
@@ -3248,7 +3236,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s" s="6">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="3"/>
@@ -3259,10 +3247,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s" s="6">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C5" t="s" s="7">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="4"/>
@@ -3272,7 +3260,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s" s="6">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="3"/>
@@ -3283,7 +3271,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s" s="6">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" s="3"/>
@@ -3294,7 +3282,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s" s="6">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="3"/>
@@ -3305,10 +3293,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s" s="6">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C9" t="s" s="7">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="4"/>
@@ -3318,11 +3306,9 @@
         <v>9</v>
       </c>
       <c r="B10" t="s" s="6">
-        <v>155</v>
-      </c>
-      <c r="C10" t="s" s="7">
-        <v>156</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="C10" s="11"/>
       <c r="D10" s="3"/>
       <c r="E10" s="4"/>
     </row>
@@ -3331,7 +3317,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s" s="6">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="3"/>
@@ -3342,7 +3328,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s" s="6">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="3"/>
@@ -3350,106 +3336,106 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="5">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s" s="6">
-        <v>159</v>
-      </c>
-      <c r="C13" s="11"/>
+        <v>156</v>
+      </c>
+      <c r="C13" t="s" s="7">
+        <v>157</v>
+      </c>
       <c r="D13" s="3"/>
       <c r="E13" s="4"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="5">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s" s="6">
-        <v>160</v>
-      </c>
-      <c r="C14" t="s" s="7">
-        <v>161</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="C14" s="13"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="5">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s" s="6">
-        <v>162</v>
-      </c>
-      <c r="C15" s="13"/>
+        <v>159</v>
+      </c>
+      <c r="C15" t="s" s="7">
+        <v>160</v>
+      </c>
       <c r="D15" s="3"/>
       <c r="E15" s="4"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="5">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s" s="6">
-        <v>163</v>
-      </c>
-      <c r="C16" t="s" s="7">
-        <v>164</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="C16" s="13"/>
       <c r="D16" s="3"/>
       <c r="E16" s="4"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="5">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s" s="6">
-        <v>165</v>
-      </c>
-      <c r="C17" s="13"/>
+        <v>162</v>
+      </c>
+      <c r="C17" t="s" s="7">
+        <v>163</v>
+      </c>
       <c r="D17" s="3"/>
       <c r="E17" s="4"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="5">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s" s="6">
-        <v>166</v>
-      </c>
-      <c r="C18" t="s" s="7">
-        <v>167</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="C18" s="11"/>
       <c r="D18" s="3"/>
       <c r="E18" s="4"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="5">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s" s="6">
-        <v>168</v>
-      </c>
-      <c r="C19" s="13"/>
+        <v>165</v>
+      </c>
+      <c r="C19" s="11"/>
       <c r="D19" s="3"/>
       <c r="E19" s="4"/>
     </row>
     <row r="20" ht="12.6" customHeight="1">
       <c r="A20" s="5">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s" s="6">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C20" t="s" s="7">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="4"/>
     </row>
     <row r="21" ht="12.6" customHeight="1">
       <c r="A21" s="5">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s" s="6">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="3"/>
@@ -3457,23 +3443,23 @@
     </row>
     <row r="22" ht="12.6" customHeight="1">
       <c r="A22" s="5">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s" s="6">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C22" t="s" s="7">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="4"/>
     </row>
     <row r="23" ht="12.6" customHeight="1">
       <c r="A23" s="5">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B23" t="s" s="6">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="3"/>
@@ -3481,10 +3467,10 @@
     </row>
     <row r="24" ht="12.6" customHeight="1">
       <c r="A24" s="5">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B24" t="s" s="6">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="3"/>
@@ -3492,10 +3478,10 @@
     </row>
     <row r="25" ht="12.6" customHeight="1">
       <c r="A25" s="5">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B25" t="s" s="6">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C25" s="13"/>
       <c r="D25" s="3"/>
@@ -3503,10 +3489,10 @@
     </row>
     <row r="26" ht="12.6" customHeight="1">
       <c r="A26" s="5">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s" s="6">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C26" s="13"/>
       <c r="D26" s="3"/>
@@ -3514,23 +3500,23 @@
     </row>
     <row r="27" ht="12.6" customHeight="1">
       <c r="A27" s="5">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B27" t="s" s="6">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C27" t="s" s="7">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="4"/>
     </row>
     <row r="28" ht="12.6" customHeight="1">
       <c r="A28" s="5">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s" s="6">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="3"/>
@@ -3538,10 +3524,10 @@
     </row>
     <row r="29" ht="12.6" customHeight="1">
       <c r="A29" s="5">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s" s="6">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C29" s="13"/>
       <c r="D29" s="3"/>
@@ -3552,12 +3538,12 @@
     <mergeCell ref="C5:C8"/>
     <mergeCell ref="C2:C4"/>
     <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="C15:C16"/>
     <mergeCell ref="C22:C26"/>
     <mergeCell ref="C27:C29"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C9:C12"/>
+    <mergeCell ref="C17:C19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
added frontend catgeory in both causes and solution sections
</commit_message>
<xml_diff>
--- a/Extracted_Data(MAS).xlsx
+++ b/Extracted_Data(MAS).xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="183">
   <si>
     <t>#ID</t>
   </si>
@@ -330,15 +330,21 @@
     <t>Missing Documentation (5)</t>
   </si>
   <si>
+    <t>User interface Problem (2)</t>
+  </si>
+  <si>
     <t>Frontend Problem (3)</t>
   </si>
   <si>
-    <t>Infrastructure Problem (9)</t>
+    <t>Output problem (1)</t>
   </si>
   <si>
     <t>Deployment Problem (3)</t>
   </si>
   <si>
+    <t>Infrastructure Problem (6)</t>
+  </si>
+  <si>
     <t>File System Handling Problem (1)</t>
   </si>
   <si>
@@ -466,6 +472,15 @@
   </si>
   <si>
     <t>Update Environment Configuration (13)</t>
+  </si>
+  <si>
+    <t>Enhance UI Display (2)</t>
+  </si>
+  <si>
+    <t>Improve Frontend  (3)</t>
+  </si>
+  <si>
+    <t>Enhance UI Interaction (1)</t>
   </si>
   <si>
     <t>Enhance Exception Handling (19)</t>
@@ -508,13 +523,10 @@
     <t>Optimize Message Handling (17)</t>
   </si>
   <si>
-    <t>Improve Frontend (3)</t>
-  </si>
-  <si>
-    <t>Optimize Infrastructure (50)</t>
-  </si>
-  <si>
     <t>Database Compatibility (6)</t>
+  </si>
+  <si>
+    <t>Optimize Infrastructure (47)</t>
   </si>
   <si>
     <t>Optimize Memory Management (41)</t>
@@ -2614,7 +2626,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultColWidth="12.8333" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" style="12" customWidth="1"/>
@@ -2845,7 +2857,9 @@
       <c r="B19" t="s" s="6">
         <v>108</v>
       </c>
-      <c r="C19" s="11"/>
+      <c r="C19" t="s" s="7">
+        <v>109</v>
+      </c>
       <c r="D19" s="3"/>
       <c r="E19" s="4"/>
     </row>
@@ -2854,7 +2868,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s" s="6">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C20" s="11"/>
       <c r="D20" s="3"/>
@@ -2865,11 +2879,9 @@
         <v>20</v>
       </c>
       <c r="B21" t="s" s="6">
-        <v>110</v>
-      </c>
-      <c r="C21" t="s" s="7">
         <v>111</v>
       </c>
+      <c r="C21" s="11"/>
       <c r="D21" s="3"/>
       <c r="E21" s="4"/>
     </row>
@@ -2880,16 +2892,18 @@
       <c r="B22" t="s" s="6">
         <v>112</v>
       </c>
-      <c r="C22" s="13"/>
+      <c r="C22" t="s" s="7">
+        <v>113</v>
+      </c>
       <c r="D22" s="3"/>
       <c r="E22" s="4"/>
     </row>
-    <row r="23" ht="12.6" customHeight="1">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="5">
         <v>22</v>
       </c>
       <c r="B23" t="s" s="6">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="3"/>
@@ -2900,11 +2914,9 @@
         <v>23</v>
       </c>
       <c r="B24" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C24" t="s" s="7">
         <v>115</v>
       </c>
+      <c r="C24" s="13"/>
       <c r="D24" s="3"/>
       <c r="E24" s="4"/>
     </row>
@@ -2915,7 +2927,9 @@
       <c r="B25" t="s" s="6">
         <v>116</v>
       </c>
-      <c r="C25" s="13"/>
+      <c r="C25" t="s" s="7">
+        <v>117</v>
+      </c>
       <c r="D25" s="3"/>
       <c r="E25" s="4"/>
     </row>
@@ -2924,11 +2938,9 @@
         <v>25</v>
       </c>
       <c r="B26" t="s" s="6">
-        <v>117</v>
-      </c>
-      <c r="C26" t="s" s="7">
         <v>118</v>
       </c>
+      <c r="C26" s="13"/>
       <c r="D26" s="3"/>
       <c r="E26" s="4"/>
     </row>
@@ -2939,7 +2951,9 @@
       <c r="B27" t="s" s="6">
         <v>119</v>
       </c>
-      <c r="C27" s="13"/>
+      <c r="C27" t="s" s="7">
+        <v>120</v>
+      </c>
       <c r="D27" s="3"/>
       <c r="E27" s="4"/>
     </row>
@@ -2948,7 +2962,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s" s="6">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="3"/>
@@ -2959,7 +2973,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s" s="6">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C29" s="13"/>
       <c r="D29" s="3"/>
@@ -2970,11 +2984,9 @@
         <v>29</v>
       </c>
       <c r="B30" t="s" s="6">
-        <v>122</v>
-      </c>
-      <c r="C30" t="s" s="7">
         <v>123</v>
       </c>
+      <c r="C30" s="13"/>
       <c r="D30" s="3"/>
       <c r="E30" s="4"/>
     </row>
@@ -2985,7 +2997,9 @@
       <c r="B31" t="s" s="6">
         <v>124</v>
       </c>
-      <c r="C31" s="13"/>
+      <c r="C31" t="s" s="7">
+        <v>125</v>
+      </c>
       <c r="D31" s="3"/>
       <c r="E31" s="4"/>
     </row>
@@ -2994,11 +3008,9 @@
         <v>31</v>
       </c>
       <c r="B32" t="s" s="6">
-        <v>125</v>
-      </c>
-      <c r="C32" t="s" s="7">
         <v>126</v>
       </c>
+      <c r="C32" s="13"/>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
     </row>
@@ -3009,7 +3021,9 @@
       <c r="B33" t="s" s="6">
         <v>127</v>
       </c>
-      <c r="C33" s="13"/>
+      <c r="C33" t="s" s="7">
+        <v>128</v>
+      </c>
       <c r="D33" s="3"/>
       <c r="E33" s="4"/>
     </row>
@@ -3018,7 +3032,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s" s="6">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C34" s="13"/>
       <c r="D34" s="3"/>
@@ -3029,7 +3043,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s" s="6">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C35" s="13"/>
       <c r="D35" s="3"/>
@@ -3040,11 +3054,9 @@
         <v>35</v>
       </c>
       <c r="B36" t="s" s="6">
-        <v>130</v>
-      </c>
-      <c r="C36" t="s" s="7">
         <v>131</v>
       </c>
+      <c r="C36" s="13"/>
       <c r="D36" s="3"/>
       <c r="E36" s="4"/>
     </row>
@@ -3055,7 +3067,9 @@
       <c r="B37" t="s" s="6">
         <v>132</v>
       </c>
-      <c r="C37" s="13"/>
+      <c r="C37" t="s" s="7">
+        <v>133</v>
+      </c>
       <c r="D37" s="3"/>
       <c r="E37" s="4"/>
     </row>
@@ -3064,7 +3078,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s" s="6">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C38" s="13"/>
       <c r="D38" s="3"/>
@@ -3075,7 +3089,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s" s="6">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C39" s="13"/>
       <c r="D39" s="3"/>
@@ -3086,7 +3100,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s" s="6">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C40" s="13"/>
       <c r="D40" s="3"/>
@@ -3097,7 +3111,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s" s="6">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C41" s="13"/>
       <c r="D41" s="3"/>
@@ -3108,7 +3122,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s" s="6">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C42" s="13"/>
       <c r="D42" s="3"/>
@@ -3119,7 +3133,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s" s="6">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C43" s="13"/>
       <c r="D43" s="3"/>
@@ -3130,7 +3144,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s" s="6">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C44" s="13"/>
       <c r="D44" s="3"/>
@@ -3141,7 +3155,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s" s="6">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C45" s="13"/>
       <c r="D45" s="3"/>
@@ -3151,28 +3165,40 @@
       <c r="A46" s="5">
         <v>45</v>
       </c>
-      <c r="B46" t="s" s="14">
-        <v>141</v>
+      <c r="B46" t="s" s="6">
+        <v>142</v>
       </c>
       <c r="C46" s="13"/>
       <c r="D46" s="3"/>
       <c r="E46" s="4"/>
     </row>
+    <row r="47" ht="12.6" customHeight="1">
+      <c r="A47" s="5">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s" s="14">
+        <v>143</v>
+      </c>
+      <c r="C47" s="13"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="C12:C14"/>
-    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="C27:C30"/>
     <mergeCell ref="C4:C6"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="C9:C11"/>
-    <mergeCell ref="C36:C46"/>
-    <mergeCell ref="C32:C35"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C21:C23"/>
+    <mergeCell ref="C37:C47"/>
+    <mergeCell ref="C33:C36"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="C22:C24"/>
     <mergeCell ref="C15:C16"/>
-    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="C31:C32"/>
     <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C17:C20"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="C17:C18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
@@ -3184,7 +3210,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="12.8333" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" style="15" customWidth="1"/>
@@ -3212,10 +3238,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s" s="6">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C2" t="s" s="7">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
@@ -3225,7 +3251,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="6">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="3"/>
@@ -3236,7 +3262,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s" s="6">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="3"/>
@@ -3247,10 +3273,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s" s="6">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C5" t="s" s="7">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="4"/>
@@ -3260,7 +3286,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s" s="6">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="3"/>
@@ -3271,7 +3297,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s" s="6">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" s="3"/>
@@ -3282,7 +3308,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s" s="6">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="3"/>
@@ -3293,10 +3319,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s" s="6">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C9" t="s" s="7">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="4"/>
@@ -3306,7 +3332,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s" s="6">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="3"/>
@@ -3317,9 +3343,11 @@
         <v>10</v>
       </c>
       <c r="B11" t="s" s="6">
-        <v>154</v>
-      </c>
-      <c r="C11" s="11"/>
+        <v>156</v>
+      </c>
+      <c r="C11" t="s" s="7">
+        <v>157</v>
+      </c>
       <c r="D11" s="3"/>
       <c r="E11" s="4"/>
     </row>
@@ -3328,7 +3356,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s" s="6">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="3"/>
@@ -3339,11 +3367,9 @@
         <v>12</v>
       </c>
       <c r="B13" t="s" s="6">
-        <v>156</v>
-      </c>
-      <c r="C13" t="s" s="7">
-        <v>157</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="C13" s="11"/>
       <c r="D13" s="3"/>
       <c r="E13" s="4"/>
     </row>
@@ -3352,9 +3378,9 @@
         <v>13</v>
       </c>
       <c r="B14" t="s" s="6">
-        <v>158</v>
-      </c>
-      <c r="C14" s="13"/>
+        <v>160</v>
+      </c>
+      <c r="C14" s="11"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
     </row>
@@ -3363,10 +3389,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s" s="6">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C15" t="s" s="7">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="4"/>
@@ -3376,7 +3402,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s" s="6">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="3"/>
@@ -3387,10 +3413,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s" s="6">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C17" t="s" s="7">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="4"/>
@@ -3400,9 +3426,9 @@
         <v>17</v>
       </c>
       <c r="B18" t="s" s="6">
-        <v>164</v>
-      </c>
-      <c r="C18" s="11"/>
+        <v>166</v>
+      </c>
+      <c r="C18" s="13"/>
       <c r="D18" s="3"/>
       <c r="E18" s="4"/>
     </row>
@@ -3411,22 +3437,22 @@
         <v>18</v>
       </c>
       <c r="B19" t="s" s="6">
-        <v>165</v>
-      </c>
-      <c r="C19" s="11"/>
+        <v>167</v>
+      </c>
+      <c r="C19" t="s" s="7">
+        <v>168</v>
+      </c>
       <c r="D19" s="3"/>
       <c r="E19" s="4"/>
     </row>
-    <row r="20" ht="12.6" customHeight="1">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="5">
         <v>19</v>
       </c>
       <c r="B20" t="s" s="6">
-        <v>166</v>
-      </c>
-      <c r="C20" t="s" s="7">
-        <v>167</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="C20" s="11"/>
       <c r="D20" s="3"/>
       <c r="E20" s="4"/>
     </row>
@@ -3435,9 +3461,11 @@
         <v>20</v>
       </c>
       <c r="B21" t="s" s="6">
-        <v>168</v>
-      </c>
-      <c r="C21" s="13"/>
+        <v>170</v>
+      </c>
+      <c r="C21" t="s" s="7">
+        <v>171</v>
+      </c>
       <c r="D21" s="3"/>
       <c r="E21" s="4"/>
     </row>
@@ -3446,11 +3474,9 @@
         <v>21</v>
       </c>
       <c r="B22" t="s" s="6">
-        <v>169</v>
-      </c>
-      <c r="C22" t="s" s="7">
-        <v>170</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="C22" s="13"/>
       <c r="D22" s="3"/>
       <c r="E22" s="4"/>
     </row>
@@ -3459,9 +3485,11 @@
         <v>22</v>
       </c>
       <c r="B23" t="s" s="6">
-        <v>171</v>
-      </c>
-      <c r="C23" s="13"/>
+        <v>173</v>
+      </c>
+      <c r="C23" t="s" s="7">
+        <v>174</v>
+      </c>
       <c r="D23" s="3"/>
       <c r="E23" s="4"/>
     </row>
@@ -3470,7 +3498,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s" s="6">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="3"/>
@@ -3481,7 +3509,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s" s="6">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C25" s="13"/>
       <c r="D25" s="3"/>
@@ -3492,7 +3520,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s" s="6">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C26" s="13"/>
       <c r="D26" s="3"/>
@@ -3503,11 +3531,9 @@
         <v>26</v>
       </c>
       <c r="B27" t="s" s="6">
-        <v>175</v>
-      </c>
-      <c r="C27" t="s" s="7">
-        <v>176</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="C27" s="13"/>
       <c r="D27" s="3"/>
       <c r="E27" s="4"/>
     </row>
@@ -3516,9 +3542,11 @@
         <v>27</v>
       </c>
       <c r="B28" t="s" s="6">
-        <v>177</v>
-      </c>
-      <c r="C28" s="13"/>
+        <v>179</v>
+      </c>
+      <c r="C28" t="s" s="7">
+        <v>180</v>
+      </c>
       <c r="D28" s="3"/>
       <c r="E28" s="4"/>
     </row>
@@ -3527,23 +3555,35 @@
         <v>28</v>
       </c>
       <c r="B29" t="s" s="6">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C29" s="13"/>
       <c r="D29" s="3"/>
       <c r="E29" s="4"/>
     </row>
+    <row r="30" ht="12.6" customHeight="1">
+      <c r="A30" s="5">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s" s="6">
+        <v>182</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="C5:C8"/>
     <mergeCell ref="C2:C4"/>
-    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C23:C27"/>
+    <mergeCell ref="C28:C30"/>
     <mergeCell ref="C15:C16"/>
-    <mergeCell ref="C22:C26"/>
-    <mergeCell ref="C27:C29"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="C9:C12"/>
-    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="C9:C10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
Update value of proformance issues
</commit_message>
<xml_diff>
--- a/Extracted_Data(MAS).xlsx
+++ b/Extracted_Data(MAS).xlsx
@@ -210,13 +210,13 @@
     <t>Incomplete Response (12)</t>
   </si>
   <si>
+    <t>Response Delay (10)</t>
+  </si>
+  <si>
+    <t>Performance Issues (19)</t>
+  </si>
+  <si>
     <t>Inefficient Execution (9)</t>
-  </si>
-  <si>
-    <t>Performance Issues (18)</t>
-  </si>
-  <si>
-    <t>Response Delay (9)</t>
   </si>
   <si>
     <t>Unhandled Exception (7)</t>
@@ -735,7 +735,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -771,6 +771,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
@@ -2469,7 +2472,7 @@
       <c r="A55" s="5">
         <v>54</v>
       </c>
-      <c r="B55" t="s" s="6">
+      <c r="B55" t="s" s="12">
         <v>67</v>
       </c>
       <c r="C55" s="11"/>
@@ -2629,11 +2632,11 @@
   <dimension ref="A1:E47"/>
   <sheetFormatPr defaultColWidth="12.8333" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="6" style="12" customWidth="1"/>
-    <col min="2" max="2" width="48" style="12" customWidth="1"/>
-    <col min="3" max="3" width="36" style="12" customWidth="1"/>
-    <col min="4" max="5" width="12.6719" style="12" customWidth="1"/>
-    <col min="6" max="16384" width="12.8516" style="12" customWidth="1"/>
+    <col min="1" max="1" width="6" style="13" customWidth="1"/>
+    <col min="2" max="2" width="48" style="13" customWidth="1"/>
+    <col min="3" max="3" width="36" style="13" customWidth="1"/>
+    <col min="4" max="5" width="12.6719" style="13" customWidth="1"/>
+    <col min="6" max="16384" width="12.8516" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -2693,7 +2696,7 @@
       <c r="B5" t="s" s="6">
         <v>89</v>
       </c>
-      <c r="C5" s="13"/>
+      <c r="C5" s="14"/>
       <c r="D5" s="3"/>
       <c r="E5" s="4"/>
     </row>
@@ -2704,7 +2707,7 @@
       <c r="B6" t="s" s="6">
         <v>90</v>
       </c>
-      <c r="C6" s="13"/>
+      <c r="C6" s="14"/>
       <c r="D6" s="3"/>
       <c r="E6" s="4"/>
     </row>
@@ -2728,7 +2731,7 @@
       <c r="B8" t="s" s="6">
         <v>93</v>
       </c>
-      <c r="C8" s="13"/>
+      <c r="C8" s="14"/>
       <c r="D8" s="3"/>
       <c r="E8" s="4"/>
     </row>
@@ -2752,7 +2755,7 @@
       <c r="B10" t="s" s="6">
         <v>96</v>
       </c>
-      <c r="C10" s="13"/>
+      <c r="C10" s="14"/>
       <c r="D10" s="3"/>
       <c r="E10" s="4"/>
     </row>
@@ -2763,7 +2766,7 @@
       <c r="B11" t="s" s="6">
         <v>97</v>
       </c>
-      <c r="C11" s="13"/>
+      <c r="C11" s="14"/>
       <c r="D11" s="3"/>
       <c r="E11" s="4"/>
     </row>
@@ -2787,7 +2790,7 @@
       <c r="B13" t="s" s="6">
         <v>100</v>
       </c>
-      <c r="C13" s="13"/>
+      <c r="C13" s="14"/>
       <c r="D13" s="3"/>
       <c r="E13" s="4"/>
     </row>
@@ -2798,7 +2801,7 @@
       <c r="B14" t="s" s="6">
         <v>101</v>
       </c>
-      <c r="C14" s="13"/>
+      <c r="C14" s="14"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
     </row>
@@ -2822,7 +2825,7 @@
       <c r="B16" t="s" s="6">
         <v>104</v>
       </c>
-      <c r="C16" s="13"/>
+      <c r="C16" s="14"/>
       <c r="D16" s="3"/>
       <c r="E16" s="4"/>
     </row>
@@ -2905,7 +2908,7 @@
       <c r="B23" t="s" s="6">
         <v>114</v>
       </c>
-      <c r="C23" s="13"/>
+      <c r="C23" s="14"/>
       <c r="D23" s="3"/>
       <c r="E23" s="4"/>
     </row>
@@ -2916,7 +2919,7 @@
       <c r="B24" t="s" s="6">
         <v>115</v>
       </c>
-      <c r="C24" s="13"/>
+      <c r="C24" s="14"/>
       <c r="D24" s="3"/>
       <c r="E24" s="4"/>
     </row>
@@ -2940,7 +2943,7 @@
       <c r="B26" t="s" s="6">
         <v>118</v>
       </c>
-      <c r="C26" s="13"/>
+      <c r="C26" s="14"/>
       <c r="D26" s="3"/>
       <c r="E26" s="4"/>
     </row>
@@ -2964,7 +2967,7 @@
       <c r="B28" t="s" s="6">
         <v>121</v>
       </c>
-      <c r="C28" s="13"/>
+      <c r="C28" s="14"/>
       <c r="D28" s="3"/>
       <c r="E28" s="4"/>
     </row>
@@ -2975,7 +2978,7 @@
       <c r="B29" t="s" s="6">
         <v>122</v>
       </c>
-      <c r="C29" s="13"/>
+      <c r="C29" s="14"/>
       <c r="D29" s="3"/>
       <c r="E29" s="4"/>
     </row>
@@ -2986,7 +2989,7 @@
       <c r="B30" t="s" s="6">
         <v>123</v>
       </c>
-      <c r="C30" s="13"/>
+      <c r="C30" s="14"/>
       <c r="D30" s="3"/>
       <c r="E30" s="4"/>
     </row>
@@ -3010,7 +3013,7 @@
       <c r="B32" t="s" s="6">
         <v>126</v>
       </c>
-      <c r="C32" s="13"/>
+      <c r="C32" s="14"/>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
     </row>
@@ -3034,7 +3037,7 @@
       <c r="B34" t="s" s="6">
         <v>129</v>
       </c>
-      <c r="C34" s="13"/>
+      <c r="C34" s="14"/>
       <c r="D34" s="3"/>
       <c r="E34" s="4"/>
     </row>
@@ -3045,7 +3048,7 @@
       <c r="B35" t="s" s="6">
         <v>130</v>
       </c>
-      <c r="C35" s="13"/>
+      <c r="C35" s="14"/>
       <c r="D35" s="3"/>
       <c r="E35" s="4"/>
     </row>
@@ -3056,7 +3059,7 @@
       <c r="B36" t="s" s="6">
         <v>131</v>
       </c>
-      <c r="C36" s="13"/>
+      <c r="C36" s="14"/>
       <c r="D36" s="3"/>
       <c r="E36" s="4"/>
     </row>
@@ -3080,7 +3083,7 @@
       <c r="B38" t="s" s="6">
         <v>134</v>
       </c>
-      <c r="C38" s="13"/>
+      <c r="C38" s="14"/>
       <c r="D38" s="3"/>
       <c r="E38" s="4"/>
     </row>
@@ -3091,7 +3094,7 @@
       <c r="B39" t="s" s="6">
         <v>135</v>
       </c>
-      <c r="C39" s="13"/>
+      <c r="C39" s="14"/>
       <c r="D39" s="3"/>
       <c r="E39" s="4"/>
     </row>
@@ -3102,7 +3105,7 @@
       <c r="B40" t="s" s="6">
         <v>136</v>
       </c>
-      <c r="C40" s="13"/>
+      <c r="C40" s="14"/>
       <c r="D40" s="3"/>
       <c r="E40" s="4"/>
     </row>
@@ -3113,7 +3116,7 @@
       <c r="B41" t="s" s="6">
         <v>137</v>
       </c>
-      <c r="C41" s="13"/>
+      <c r="C41" s="14"/>
       <c r="D41" s="3"/>
       <c r="E41" s="4"/>
     </row>
@@ -3124,7 +3127,7 @@
       <c r="B42" t="s" s="6">
         <v>138</v>
       </c>
-      <c r="C42" s="13"/>
+      <c r="C42" s="14"/>
       <c r="D42" s="3"/>
       <c r="E42" s="4"/>
     </row>
@@ -3135,7 +3138,7 @@
       <c r="B43" t="s" s="6">
         <v>139</v>
       </c>
-      <c r="C43" s="13"/>
+      <c r="C43" s="14"/>
       <c r="D43" s="3"/>
       <c r="E43" s="4"/>
     </row>
@@ -3146,7 +3149,7 @@
       <c r="B44" t="s" s="6">
         <v>140</v>
       </c>
-      <c r="C44" s="13"/>
+      <c r="C44" s="14"/>
       <c r="D44" s="3"/>
       <c r="E44" s="4"/>
     </row>
@@ -3157,7 +3160,7 @@
       <c r="B45" t="s" s="6">
         <v>141</v>
       </c>
-      <c r="C45" s="13"/>
+      <c r="C45" s="14"/>
       <c r="D45" s="3"/>
       <c r="E45" s="4"/>
     </row>
@@ -3168,7 +3171,7 @@
       <c r="B46" t="s" s="6">
         <v>142</v>
       </c>
-      <c r="C46" s="13"/>
+      <c r="C46" s="14"/>
       <c r="D46" s="3"/>
       <c r="E46" s="4"/>
     </row>
@@ -3176,10 +3179,10 @@
       <c r="A47" s="5">
         <v>46</v>
       </c>
-      <c r="B47" t="s" s="14">
+      <c r="B47" t="s" s="15">
         <v>143</v>
       </c>
-      <c r="C47" s="13"/>
+      <c r="C47" s="14"/>
       <c r="D47" s="3"/>
       <c r="E47" s="4"/>
     </row>
@@ -3213,11 +3216,11 @@
   <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="12.8333" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="6" style="15" customWidth="1"/>
-    <col min="2" max="2" width="48" style="15" customWidth="1"/>
-    <col min="3" max="3" width="36" style="15" customWidth="1"/>
-    <col min="4" max="5" width="12.6719" style="15" customWidth="1"/>
-    <col min="6" max="16384" width="12.8516" style="15" customWidth="1"/>
+    <col min="1" max="1" width="6" style="16" customWidth="1"/>
+    <col min="2" max="2" width="48" style="16" customWidth="1"/>
+    <col min="3" max="3" width="36" style="16" customWidth="1"/>
+    <col min="4" max="5" width="12.6719" style="16" customWidth="1"/>
+    <col min="6" max="16384" width="12.8516" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -3253,7 +3256,7 @@
       <c r="B3" t="s" s="6">
         <v>146</v>
       </c>
-      <c r="C3" s="13"/>
+      <c r="C3" s="14"/>
       <c r="D3" s="3"/>
       <c r="E3" s="4"/>
     </row>
@@ -3264,7 +3267,7 @@
       <c r="B4" t="s" s="6">
         <v>147</v>
       </c>
-      <c r="C4" s="13"/>
+      <c r="C4" s="14"/>
       <c r="D4" s="3"/>
       <c r="E4" s="4"/>
     </row>
@@ -3288,7 +3291,7 @@
       <c r="B6" t="s" s="6">
         <v>150</v>
       </c>
-      <c r="C6" s="13"/>
+      <c r="C6" s="14"/>
       <c r="D6" s="3"/>
       <c r="E6" s="4"/>
     </row>
@@ -3299,7 +3302,7 @@
       <c r="B7" t="s" s="6">
         <v>151</v>
       </c>
-      <c r="C7" s="13"/>
+      <c r="C7" s="14"/>
       <c r="D7" s="3"/>
       <c r="E7" s="4"/>
     </row>
@@ -3310,7 +3313,7 @@
       <c r="B8" t="s" s="6">
         <v>152</v>
       </c>
-      <c r="C8" s="13"/>
+      <c r="C8" s="14"/>
       <c r="D8" s="3"/>
       <c r="E8" s="4"/>
     </row>
@@ -3404,7 +3407,7 @@
       <c r="B16" t="s" s="6">
         <v>163</v>
       </c>
-      <c r="C16" s="13"/>
+      <c r="C16" s="14"/>
       <c r="D16" s="3"/>
       <c r="E16" s="4"/>
     </row>
@@ -3428,7 +3431,7 @@
       <c r="B18" t="s" s="6">
         <v>166</v>
       </c>
-      <c r="C18" s="13"/>
+      <c r="C18" s="14"/>
       <c r="D18" s="3"/>
       <c r="E18" s="4"/>
     </row>
@@ -3476,7 +3479,7 @@
       <c r="B22" t="s" s="6">
         <v>172</v>
       </c>
-      <c r="C22" s="13"/>
+      <c r="C22" s="14"/>
       <c r="D22" s="3"/>
       <c r="E22" s="4"/>
     </row>
@@ -3500,7 +3503,7 @@
       <c r="B24" t="s" s="6">
         <v>175</v>
       </c>
-      <c r="C24" s="13"/>
+      <c r="C24" s="14"/>
       <c r="D24" s="3"/>
       <c r="E24" s="4"/>
     </row>
@@ -3511,7 +3514,7 @@
       <c r="B25" t="s" s="6">
         <v>176</v>
       </c>
-      <c r="C25" s="13"/>
+      <c r="C25" s="14"/>
       <c r="D25" s="3"/>
       <c r="E25" s="4"/>
     </row>
@@ -3522,7 +3525,7 @@
       <c r="B26" t="s" s="6">
         <v>177</v>
       </c>
-      <c r="C26" s="13"/>
+      <c r="C26" s="14"/>
       <c r="D26" s="3"/>
       <c r="E26" s="4"/>
     </row>
@@ -3533,7 +3536,7 @@
       <c r="B27" t="s" s="6">
         <v>178</v>
       </c>
-      <c r="C27" s="13"/>
+      <c r="C27" s="14"/>
       <c r="D27" s="3"/>
       <c r="E27" s="4"/>
     </row>
@@ -3557,7 +3560,7 @@
       <c r="B29" t="s" s="6">
         <v>181</v>
       </c>
-      <c r="C29" s="13"/>
+      <c r="C29" s="14"/>
       <c r="D29" s="3"/>
       <c r="E29" s="4"/>
     </row>
@@ -3568,7 +3571,7 @@
       <c r="B30" t="s" s="6">
         <v>182</v>
       </c>
-      <c r="C30" s="13"/>
+      <c r="C30" s="14"/>
       <c r="D30" s="3"/>
       <c r="E30" s="4"/>
     </row>

</xml_diff>

<commit_message>
update categgories name in solution section
</commit_message>
<xml_diff>
--- a/Extracted_Data(MAS).xlsx
+++ b/Extracted_Data(MAS).xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="182">
   <si>
     <t>#ID</t>
   </si>
@@ -453,10 +453,10 @@
     <t>Adjust Agent Initialization (29)</t>
   </si>
   <si>
-    <t>Optimize Agent Creation (18)</t>
-  </si>
-  <si>
-    <t>Configure Agent Dependencies (8)</t>
+    <t>Correct Agent Initialization (18)</t>
+  </si>
+  <si>
+    <t>Configure Agent Integration (8)</t>
   </si>
   <si>
     <t>Refine Prompt (4)</t>
@@ -508,10 +508,10 @@
     <t>Add Documentation (6)</t>
   </si>
   <si>
-    <t>Modify Documentation (13)</t>
-  </si>
-  <si>
-    <t>Modify Description (7)</t>
+    <t>Improve Documentation (13)</t>
+  </si>
+  <si>
+    <t>Modify Documentation (7)</t>
   </si>
   <si>
     <t>Optimize Inter-agent Communication (16)</t>
@@ -559,16 +559,13 @@
     <t>Optimize Sequential Execution (10)</t>
   </si>
   <si>
-    <t>Fix Version Compatibility (27)</t>
+    <t>Fix Version Compatibility (29)</t>
   </si>
   <si>
     <t>Update Dependencies (31)</t>
   </si>
   <si>
     <t>Add Missing Dependency (2)</t>
-  </si>
-  <si>
-    <t>Version Mismatch (2)</t>
   </si>
 </sst>
 </file>
@@ -3213,7 +3210,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultColWidth="12.8333" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" style="16" customWidth="1"/>
@@ -3564,17 +3561,6 @@
       <c r="D29" s="3"/>
       <c r="E29" s="4"/>
     </row>
-    <row r="30" ht="12.6" customHeight="1">
-      <c r="A30" s="5">
-        <v>29</v>
-      </c>
-      <c r="B30" t="s" s="6">
-        <v>182</v>
-      </c>
-      <c r="C30" s="14"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="4"/>
-    </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="C5:C8"/>
@@ -3582,7 +3568,7 @@
     <mergeCell ref="C21:C22"/>
     <mergeCell ref="C17:C18"/>
     <mergeCell ref="C23:C27"/>
-    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="C28:C29"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="C11:C14"/>
     <mergeCell ref="C19:C20"/>

</xml_diff>